<commit_message>
Update FASTA reporting artifacts
</commit_message>
<xml_diff>
--- a/reports/FASTA_ML_Results_2026-06-17.xlsx
+++ b/reports/FASTA_ML_Results_2026-06-17.xlsx
@@ -43,7 +43,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="FF006272"/>
+      <color rgb="FFFFC107"/>
       <sz val="10"/>
     </font>
     <font>
@@ -64,7 +64,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF006272"/>
+      <color rgb="FFFFC107"/>
       <sz val="11"/>
     </font>
     <font>
@@ -75,7 +75,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FF00B050"/>
+      <color rgb="FF27ae60"/>
       <sz val="10"/>
     </font>
     <font>
@@ -86,7 +86,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FFEE5a6f"/>
       <sz val="10"/>
     </font>
     <font>
@@ -94,7 +94,7 @@
       <sz val="10"/>
     </font>
     <font>
-      <color rgb="FFFF0000"/>
+      <color rgb="FFEE5a6f"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -107,17 +107,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF006272"/>
+        <fgColor rgb="FF1A2E44"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE0F0F1"/>
+        <fgColor rgb="FF2C3E50"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFF5f5f5"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +127,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor rgb="FFFFC107"/>
       </patternFill>
     </fill>
   </fills>

</xml_diff>